<commit_message>
Case a cocher excel
</commit_message>
<xml_diff>
--- a/2026_Planning_IT_BLEU.xlsx
+++ b/2026_Planning_IT_BLEU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\DSS2_IT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5195B0DD-02F8-4AC1-84F8-3D779F45853C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F7E4802-DED8-46BE-A06D-16916C612723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C705B5AA-50E9-48AD-9A1C-4B16FAE8BD48}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="133">
   <si>
     <t>Lu</t>
   </si>
@@ -618,12 +618,15 @@
   <si>
     <t>Documentation</t>
   </si>
+  <si>
+    <t>Validée</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -683,6 +686,14 @@
       <sz val="11"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="22">
@@ -813,7 +824,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -1065,7 +1076,35 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -1128,6 +1167,24 @@
     <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1137,33 +1194,39 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1179,6 +1242,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1478,7 +1558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD0E5664-ED85-44C0-B9CF-6C0ACD2C2B32}">
-  <dimension ref="A1:Q58"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="85.5703125" customWidth="1"/>
@@ -1486,30 +1566,33 @@
     <col min="3" max="17" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="C1" s="36" t="s">
+    <row r="1" spans="1:18" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="C1" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="36" t="s">
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="54" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="36" t="s">
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="38"/>
-    </row>
-    <row r="2" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="57" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="25" t="s">
         <v>76</v>
@@ -1560,7 +1643,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -1581,7 +1664,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -1602,7 +1685,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>90</v>
       </c>
@@ -1625,7 +1708,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1646,7 +1729,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>120</v>
       </c>
@@ -1667,7 +1750,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>117</v>
       </c>
@@ -1688,7 +1771,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -1709,7 +1792,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1730,7 +1813,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="4"/>
     </row>
-    <row r="11" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>72</v>
       </c>
@@ -1751,7 +1834,7 @@
       <c r="P11" s="20"/>
       <c r="Q11" s="20"/>
     </row>
-    <row r="12" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>118</v>
       </c>
@@ -1774,7 +1857,7 @@
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
     </row>
-    <row r="13" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>108</v>
       </c>
@@ -1797,7 +1880,7 @@
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
     </row>
-    <row r="14" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>109</v>
       </c>
@@ -1820,7 +1903,7 @@
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
     </row>
-    <row r="15" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>110</v>
       </c>
@@ -1843,7 +1926,7 @@
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
     </row>
-    <row r="16" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>111</v>
       </c>
@@ -2230,7 +2313,7 @@
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>103</v>
       </c>
@@ -2253,7 +2336,7 @@
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
     </row>
-    <row r="34" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>104</v>
       </c>
@@ -2276,7 +2359,7 @@
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
     </row>
-    <row r="35" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
         <v>82</v>
       </c>
@@ -2297,7 +2380,7 @@
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
     </row>
-    <row r="36" spans="1:17" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>105</v>
       </c>
@@ -2320,52 +2403,56 @@
       <c r="P36" s="11"/>
       <c r="Q36" s="1"/>
     </row>
-    <row r="37" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="41" t="s">
+    <row r="37" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="B37" s="41"/>
-      <c r="C37" s="42"/>
-      <c r="D37" s="42"/>
-      <c r="E37" s="42"/>
-      <c r="F37" s="42"/>
-      <c r="G37" s="42"/>
-      <c r="H37" s="42"/>
-      <c r="I37" s="42"/>
-      <c r="J37" s="42"/>
-      <c r="K37" s="42"/>
-      <c r="L37" s="42"/>
-      <c r="M37" s="42"/>
-      <c r="N37" s="42"/>
-      <c r="O37" s="42"/>
-      <c r="P37" s="42"/>
-      <c r="Q37" s="42"/>
-    </row>
-    <row r="38" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A38" s="43" t="s">
+      <c r="B37" s="36"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="37"/>
+      <c r="I37" s="37"/>
+      <c r="J37" s="37"/>
+      <c r="K37" s="37"/>
+      <c r="L37" s="37"/>
+      <c r="M37" s="37"/>
+      <c r="N37" s="37"/>
+      <c r="O37" s="37"/>
+      <c r="P37" s="37"/>
+      <c r="Q37" s="37"/>
+      <c r="R37" s="37"/>
+    </row>
+    <row r="38" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A38" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="B38" s="44" t="s">
+      <c r="B38" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C38" s="45"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="46"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="47"/>
-      <c r="J38" s="47"/>
-      <c r="K38" s="47"/>
-      <c r="L38" s="47"/>
-      <c r="M38" s="47"/>
-      <c r="N38" s="47"/>
-      <c r="O38" s="47"/>
-      <c r="P38" s="47"/>
-      <c r="Q38" s="48"/>
-    </row>
-    <row r="39" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A39" s="49" t="s">
+      <c r="C38" s="40"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="42"/>
+      <c r="I38" s="42"/>
+      <c r="J38" s="42"/>
+      <c r="K38" s="42"/>
+      <c r="L38" s="42"/>
+      <c r="M38" s="42"/>
+      <c r="N38" s="42"/>
+      <c r="O38" s="42"/>
+      <c r="P38" s="42"/>
+      <c r="Q38" s="58"/>
+      <c r="R38" s="61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A39" s="43" t="s">
         <v>123</v>
       </c>
       <c r="B39" s="1"/>
@@ -2383,10 +2470,13 @@
       <c r="N39" s="7"/>
       <c r="O39" s="7"/>
       <c r="P39" s="7"/>
-      <c r="Q39" s="50"/>
-    </row>
-    <row r="40" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A40" s="49" t="s">
+      <c r="Q39" s="59"/>
+      <c r="R39" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A40" s="43" t="s">
         <v>121</v>
       </c>
       <c r="B40" s="1"/>
@@ -2404,322 +2494,367 @@
       <c r="N40" s="7"/>
       <c r="O40" s="7"/>
       <c r="P40" s="7"/>
-      <c r="Q40" s="50"/>
-    </row>
-    <row r="41" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="51" t="s">
+      <c r="Q40" s="59"/>
+      <c r="R40" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="B41" s="52"/>
-      <c r="C41" s="53"/>
-      <c r="D41" s="54"/>
-      <c r="E41" s="54"/>
-      <c r="F41" s="55"/>
-      <c r="G41" s="55"/>
-      <c r="H41" s="55"/>
-      <c r="I41" s="55"/>
-      <c r="J41" s="55"/>
-      <c r="K41" s="55"/>
-      <c r="L41" s="55"/>
-      <c r="M41" s="55"/>
-      <c r="N41" s="55"/>
-      <c r="O41" s="55"/>
-      <c r="P41" s="55"/>
-      <c r="Q41" s="56"/>
-    </row>
-    <row r="42" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A42" s="43" t="s">
+      <c r="B41" s="45"/>
+      <c r="C41" s="46"/>
+      <c r="D41" s="47"/>
+      <c r="E41" s="47"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48"/>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
+      <c r="M41" s="48"/>
+      <c r="N41" s="48"/>
+      <c r="O41" s="48"/>
+      <c r="P41" s="48"/>
+      <c r="Q41" s="60"/>
+      <c r="R41" s="63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A42" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="B42" s="44" t="s">
+      <c r="B42" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C42" s="45"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46"/>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
-      <c r="M42" s="47"/>
-      <c r="N42" s="47"/>
-      <c r="O42" s="47"/>
-      <c r="P42" s="47"/>
-      <c r="Q42" s="48"/>
-    </row>
-    <row r="43" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A43" s="49" t="s">
+      <c r="C42" s="40"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="41"/>
+      <c r="G42" s="41"/>
+      <c r="H42" s="41"/>
+      <c r="I42" s="41"/>
+      <c r="J42" s="41"/>
+      <c r="K42" s="41"/>
+      <c r="L42" s="41"/>
+      <c r="M42" s="42"/>
+      <c r="N42" s="42"/>
+      <c r="O42" s="42"/>
+      <c r="P42" s="42"/>
+      <c r="Q42" s="58"/>
+      <c r="R42" s="61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A43" s="43" t="s">
         <v>124</v>
       </c>
       <c r="B43" s="1"/>
       <c r="C43" s="10"/>
       <c r="D43" s="8"/>
       <c r="E43" s="8"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="39"/>
-      <c r="I43" s="39"/>
-      <c r="J43" s="39"/>
-      <c r="K43" s="39"/>
-      <c r="L43" s="39"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="7"/>
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
       <c r="O43" s="7"/>
       <c r="P43" s="7"/>
-      <c r="Q43" s="50"/>
-    </row>
-    <row r="44" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A44" s="49" t="s">
+      <c r="Q43" s="59"/>
+      <c r="R43" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A44" s="43" t="s">
         <v>125</v>
       </c>
       <c r="B44" s="1"/>
       <c r="C44" s="10"/>
-      <c r="D44" s="39"/>
-      <c r="E44" s="39"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="8"/>
-      <c r="J44" s="39"/>
-      <c r="K44" s="39"/>
-      <c r="L44" s="39"/>
+      <c r="J44" s="7"/>
+      <c r="K44" s="7"/>
+      <c r="L44" s="7"/>
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
       <c r="O44" s="7"/>
       <c r="P44" s="7"/>
-      <c r="Q44" s="50"/>
-    </row>
-    <row r="45" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A45" s="49" t="s">
+      <c r="Q44" s="59"/>
+      <c r="R44" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A45" s="43" t="s">
         <v>126</v>
       </c>
       <c r="B45" s="1"/>
       <c r="C45" s="10"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="39"/>
-      <c r="H45" s="39"/>
-      <c r="I45" s="39"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
-      <c r="L45" s="39"/>
+      <c r="L45" s="7"/>
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
       <c r="O45" s="7"/>
       <c r="P45" s="7"/>
-      <c r="Q45" s="50"/>
-    </row>
-    <row r="46" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="51" t="s">
+      <c r="Q45" s="59"/>
+      <c r="R45" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="B46" s="52"/>
-      <c r="C46" s="53"/>
-      <c r="D46" s="57"/>
-      <c r="E46" s="54"/>
-      <c r="F46" s="57"/>
-      <c r="G46" s="57"/>
-      <c r="H46" s="57"/>
-      <c r="I46" s="57"/>
-      <c r="J46" s="57"/>
-      <c r="K46" s="57"/>
-      <c r="L46" s="57"/>
-      <c r="M46" s="55"/>
-      <c r="N46" s="55"/>
-      <c r="O46" s="55"/>
-      <c r="P46" s="55"/>
-      <c r="Q46" s="56"/>
-    </row>
-    <row r="47" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A47" s="43" t="s">
+      <c r="B46" s="45"/>
+      <c r="C46" s="46"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="47"/>
+      <c r="F46" s="48"/>
+      <c r="G46" s="48"/>
+      <c r="H46" s="48"/>
+      <c r="I46" s="48"/>
+      <c r="J46" s="48"/>
+      <c r="K46" s="48"/>
+      <c r="L46" s="48"/>
+      <c r="M46" s="48"/>
+      <c r="N46" s="48"/>
+      <c r="O46" s="48"/>
+      <c r="P46" s="48"/>
+      <c r="Q46" s="60"/>
+      <c r="R46" s="63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A47" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="B47" s="44" t="s">
+      <c r="B47" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="45"/>
-      <c r="D47" s="46"/>
-      <c r="E47" s="46"/>
-      <c r="F47" s="46"/>
-      <c r="G47" s="46"/>
-      <c r="H47" s="46"/>
-      <c r="I47" s="46"/>
-      <c r="J47" s="46"/>
-      <c r="K47" s="46"/>
-      <c r="L47" s="46"/>
-      <c r="M47" s="47"/>
-      <c r="N47" s="47"/>
-      <c r="O47" s="47"/>
-      <c r="P47" s="47"/>
-      <c r="Q47" s="48"/>
-    </row>
-    <row r="48" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A48" s="49" t="s">
+      <c r="C47" s="40"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="41"/>
+      <c r="F47" s="41"/>
+      <c r="G47" s="41"/>
+      <c r="H47" s="41"/>
+      <c r="I47" s="41"/>
+      <c r="J47" s="41"/>
+      <c r="K47" s="41"/>
+      <c r="L47" s="41"/>
+      <c r="M47" s="42"/>
+      <c r="N47" s="42"/>
+      <c r="O47" s="42"/>
+      <c r="P47" s="42"/>
+      <c r="Q47" s="58"/>
+      <c r="R47" s="61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A48" s="43" t="s">
         <v>124</v>
       </c>
       <c r="B48" s="1"/>
-      <c r="C48" s="40"/>
+      <c r="C48" s="10"/>
       <c r="D48" s="8"/>
       <c r="E48" s="8"/>
-      <c r="F48" s="39"/>
-      <c r="G48" s="39"/>
-      <c r="H48" s="39"/>
-      <c r="I48" s="39"/>
-      <c r="J48" s="39"/>
-      <c r="K48" s="39"/>
-      <c r="L48" s="39"/>
-      <c r="M48" s="39"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="7"/>
+      <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
       <c r="N48" s="7"/>
       <c r="O48" s="7"/>
       <c r="P48" s="7"/>
-      <c r="Q48" s="50"/>
-    </row>
-    <row r="49" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A49" s="49" t="s">
+      <c r="Q48" s="59"/>
+      <c r="R48" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A49" s="43" t="s">
         <v>125</v>
       </c>
       <c r="B49" s="1"/>
-      <c r="C49" s="40"/>
-      <c r="D49" s="39"/>
-      <c r="E49" s="39"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
-      <c r="H49" s="39"/>
-      <c r="I49" s="39"/>
-      <c r="J49" s="39"/>
-      <c r="K49" s="39"/>
-      <c r="L49" s="39"/>
-      <c r="M49" s="39"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
       <c r="N49" s="7"/>
       <c r="O49" s="7"/>
       <c r="P49" s="7"/>
-      <c r="Q49" s="50"/>
-    </row>
-    <row r="50" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A50" s="49" t="s">
+      <c r="Q49" s="59"/>
+      <c r="R49" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A50" s="43" t="s">
         <v>126</v>
       </c>
       <c r="B50" s="1"/>
-      <c r="C50" s="40"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="39"/>
-      <c r="F50" s="39"/>
-      <c r="G50" s="39"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
       <c r="H50" s="8"/>
-      <c r="I50" s="39"/>
-      <c r="J50" s="39"/>
-      <c r="K50" s="39"/>
-      <c r="L50" s="39"/>
-      <c r="M50" s="39"/>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
       <c r="N50" s="7"/>
       <c r="O50" s="7"/>
       <c r="P50" s="7"/>
-      <c r="Q50" s="50"/>
-    </row>
-    <row r="51" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="51" t="s">
+      <c r="Q50" s="59"/>
+      <c r="R50" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="B51" s="52"/>
-      <c r="C51" s="58"/>
-      <c r="D51" s="57"/>
-      <c r="E51" s="54"/>
-      <c r="F51" s="57"/>
-      <c r="G51" s="57"/>
-      <c r="H51" s="57"/>
-      <c r="I51" s="57"/>
-      <c r="J51" s="57"/>
-      <c r="K51" s="57"/>
-      <c r="L51" s="57"/>
-      <c r="M51" s="57"/>
-      <c r="N51" s="55"/>
-      <c r="O51" s="55"/>
-      <c r="P51" s="55"/>
-      <c r="Q51" s="56"/>
-    </row>
-    <row r="52" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="43" t="s">
+      <c r="B51" s="45"/>
+      <c r="C51" s="46"/>
+      <c r="D51" s="48"/>
+      <c r="E51" s="47"/>
+      <c r="F51" s="48"/>
+      <c r="G51" s="48"/>
+      <c r="H51" s="48"/>
+      <c r="I51" s="48"/>
+      <c r="J51" s="48"/>
+      <c r="K51" s="48"/>
+      <c r="L51" s="48"/>
+      <c r="M51" s="48"/>
+      <c r="N51" s="48"/>
+      <c r="O51" s="48"/>
+      <c r="P51" s="48"/>
+      <c r="Q51" s="60"/>
+      <c r="R51" s="63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="44" t="s">
+      <c r="B52" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="45"/>
-      <c r="D52" s="47"/>
-      <c r="E52" s="47"/>
-      <c r="F52" s="47"/>
-      <c r="G52" s="47"/>
-      <c r="H52" s="47"/>
-      <c r="I52" s="47"/>
-      <c r="J52" s="46"/>
-      <c r="K52" s="46"/>
-      <c r="L52" s="46"/>
-      <c r="M52" s="46"/>
-      <c r="N52" s="46"/>
-      <c r="O52" s="47"/>
-      <c r="P52" s="47"/>
-      <c r="Q52" s="48"/>
-    </row>
-    <row r="53" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="43" t="s">
+      <c r="C52" s="65"/>
+      <c r="D52" s="51"/>
+      <c r="E52" s="51"/>
+      <c r="F52" s="51"/>
+      <c r="G52" s="51"/>
+      <c r="H52" s="51"/>
+      <c r="I52" s="51"/>
+      <c r="J52" s="53"/>
+      <c r="K52" s="53"/>
+      <c r="L52" s="53"/>
+      <c r="M52" s="53"/>
+      <c r="N52" s="53"/>
+      <c r="O52" s="51"/>
+      <c r="P52" s="51"/>
+      <c r="Q52" s="52"/>
+      <c r="R52" s="64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="49" t="s">
         <v>75</v>
       </c>
-      <c r="B53" s="44" t="s">
+      <c r="B53" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="C53" s="45"/>
-      <c r="D53" s="47"/>
-      <c r="E53" s="47"/>
-      <c r="F53" s="47"/>
-      <c r="G53" s="47"/>
-      <c r="H53" s="47"/>
-      <c r="I53" s="47"/>
-      <c r="J53" s="46"/>
-      <c r="K53" s="46"/>
-      <c r="L53" s="46"/>
-      <c r="M53" s="46"/>
-      <c r="N53" s="46"/>
-      <c r="O53" s="47"/>
-      <c r="P53" s="47"/>
-      <c r="Q53" s="48"/>
-    </row>
-    <row r="54" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A54" s="43" t="s">
+      <c r="C53" s="65"/>
+      <c r="D53" s="51"/>
+      <c r="E53" s="51"/>
+      <c r="F53" s="51"/>
+      <c r="G53" s="51"/>
+      <c r="H53" s="51"/>
+      <c r="I53" s="51"/>
+      <c r="J53" s="53"/>
+      <c r="K53" s="53"/>
+      <c r="L53" s="53"/>
+      <c r="M53" s="53"/>
+      <c r="N53" s="53"/>
+      <c r="O53" s="51"/>
+      <c r="P53" s="51"/>
+      <c r="Q53" s="52"/>
+      <c r="R53" s="64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A54" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="B54" s="44" t="s">
+      <c r="B54" s="39" t="s">
         <v>106</v>
       </c>
-      <c r="C54" s="45"/>
-      <c r="D54" s="64"/>
-      <c r="E54" s="64"/>
-      <c r="F54" s="64"/>
-      <c r="G54" s="64"/>
-      <c r="H54" s="46"/>
-      <c r="I54" s="46"/>
-      <c r="J54" s="46"/>
-      <c r="K54" s="46"/>
-      <c r="L54" s="46"/>
-      <c r="M54" s="47"/>
-      <c r="N54" s="47"/>
-      <c r="O54" s="47"/>
-      <c r="P54" s="47"/>
-      <c r="Q54" s="48"/>
-    </row>
-    <row r="55" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A55" s="49" t="s">
+      <c r="C54" s="40"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="42"/>
+      <c r="F54" s="42"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="41"/>
+      <c r="J54" s="41"/>
+      <c r="K54" s="41"/>
+      <c r="L54" s="41"/>
+      <c r="M54" s="42"/>
+      <c r="N54" s="42"/>
+      <c r="O54" s="42"/>
+      <c r="P54" s="42"/>
+      <c r="Q54" s="58"/>
+      <c r="R54" s="61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A55" s="43" t="s">
         <v>129</v>
       </c>
       <c r="B55" s="1"/>
       <c r="C55" s="10"/>
-      <c r="D55" s="39"/>
-      <c r="E55" s="39"/>
-      <c r="F55" s="39"/>
-      <c r="G55" s="39"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
       <c r="J55" s="8"/>
@@ -2729,18 +2864,21 @@
       <c r="N55" s="7"/>
       <c r="O55" s="7"/>
       <c r="P55" s="7"/>
-      <c r="Q55" s="50"/>
-    </row>
-    <row r="56" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A56" s="49" t="s">
+      <c r="Q55" s="59"/>
+      <c r="R55" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A56" s="43" t="s">
         <v>130</v>
       </c>
       <c r="B56" s="1"/>
       <c r="C56" s="10"/>
-      <c r="D56" s="39"/>
-      <c r="E56" s="39"/>
-      <c r="F56" s="39"/>
-      <c r="G56" s="39"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
       <c r="J56" s="8"/>
@@ -2750,51 +2888,60 @@
       <c r="N56" s="7"/>
       <c r="O56" s="7"/>
       <c r="P56" s="7"/>
-      <c r="Q56" s="50"/>
-    </row>
-    <row r="57" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="51" t="s">
+      <c r="Q56" s="59"/>
+      <c r="R56" s="62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="B57" s="52"/>
-      <c r="C57" s="53"/>
-      <c r="D57" s="57"/>
-      <c r="E57" s="57"/>
-      <c r="F57" s="57"/>
-      <c r="G57" s="57"/>
-      <c r="H57" s="54"/>
-      <c r="I57" s="54"/>
-      <c r="J57" s="54"/>
-      <c r="K57" s="54"/>
-      <c r="L57" s="54"/>
-      <c r="M57" s="55"/>
-      <c r="N57" s="55"/>
-      <c r="O57" s="55"/>
-      <c r="P57" s="55"/>
-      <c r="Q57" s="56"/>
-    </row>
-    <row r="58" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="59" t="s">
+      <c r="B57" s="45"/>
+      <c r="C57" s="46"/>
+      <c r="D57" s="48"/>
+      <c r="E57" s="48"/>
+      <c r="F57" s="48"/>
+      <c r="G57" s="48"/>
+      <c r="H57" s="47"/>
+      <c r="I57" s="47"/>
+      <c r="J57" s="47"/>
+      <c r="K57" s="47"/>
+      <c r="L57" s="47"/>
+      <c r="M57" s="48"/>
+      <c r="N57" s="48"/>
+      <c r="O57" s="48"/>
+      <c r="P57" s="48"/>
+      <c r="Q57" s="60"/>
+      <c r="R57" s="63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="49" t="s">
         <v>88</v>
       </c>
-      <c r="B58" s="60" t="s">
+      <c r="B58" s="50" t="s">
         <v>106</v>
       </c>
-      <c r="C58" s="61"/>
-      <c r="D58" s="61"/>
-      <c r="E58" s="61"/>
-      <c r="F58" s="61"/>
-      <c r="G58" s="61"/>
-      <c r="H58" s="61"/>
-      <c r="I58" s="61"/>
-      <c r="J58" s="61"/>
-      <c r="K58" s="61"/>
-      <c r="L58" s="62"/>
-      <c r="M58" s="65"/>
-      <c r="N58" s="65"/>
-      <c r="O58" s="65"/>
-      <c r="P58" s="65"/>
-      <c r="Q58" s="63"/>
+      <c r="C58" s="51"/>
+      <c r="D58" s="51"/>
+      <c r="E58" s="51"/>
+      <c r="F58" s="51"/>
+      <c r="G58" s="51"/>
+      <c r="H58" s="51"/>
+      <c r="I58" s="51"/>
+      <c r="J58" s="51"/>
+      <c r="K58" s="51"/>
+      <c r="L58" s="51"/>
+      <c r="M58" s="53"/>
+      <c r="N58" s="53"/>
+      <c r="O58" s="53"/>
+      <c r="P58" s="53"/>
+      <c r="Q58" s="51"/>
+      <c r="R58" s="64" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3431,15 +3578,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="d0786592-814e-4ed5-bda0-b28f68a8b04b" xsi:nil="true"/>
@@ -3448,6 +3586,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3470,14 +3617,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{817FB5F0-447E-4669-9B86-F8C140A4747C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71EA6D1C-59E5-4E02-AAD9-E8B1E631E44A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3486,4 +3625,12 @@
     <ds:schemaRef ds:uri="2f424ab4-139f-41e4-a064-161e9e1e8920"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{817FB5F0-447E-4669-9B86-F8C140A4747C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>